<commit_message>
feat(module-4): synchronize docs and site with live Module_4_Demo.xlsx calculations and Table_VS_Range drill
</commit_message>
<xml_diff>
--- a/11_Demos_and_Workbooks/04_Tables/Module_4_Demo.xlsx
+++ b/11_Demos_and_Workbooks/04_Tables/Module_4_Demo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\courses\Data Analysis 26-27\7-Introducation to Data Fields (Excel)\11_Demos_and_Workbooks\04_Tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F7D4B77-BCFA-4FE3-B49C-F19859757186}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C422E4F4-1B91-4282-8997-AC9E26293B16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table_VS_Range " sheetId="5" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="902" uniqueCount="355">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="907" uniqueCount="360">
   <si>
     <t>OrderID</t>
   </si>
@@ -1102,14 +1102,30 @@
   </si>
   <si>
     <t>EmailDomain</t>
+  </si>
+  <si>
+    <t>InventoryValuation</t>
+  </si>
+  <si>
+    <t>GrossMarginEGP</t>
+  </si>
+  <si>
+    <t>MarkupPercentage</t>
+  </si>
+  <si>
+    <t>ReorderAlert</t>
+  </si>
+  <si>
+    <t>DeptHead</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="[$$-409]#,##0.00"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -1224,7 +1240,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1285,11 +1301,47 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="53">
+  <dxfs count="58">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="[$$-409]#,##0.00"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="[$$-409]#,##0.00"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="[$$-409]#,##0.00"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="[$$-409]#,##0.00"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="[$$-409]#,##0.00"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1307,12 +1359,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1731,13 +1777,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5A9DE322-2FCB-425C-BA76-00C4CCA9C34F}" name="Table2" displayName="Table2" ref="G6:J13" totalsRowCount="1" headerRowDxfId="47" dataDxfId="48" tableBorderDxfId="52">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5A9DE322-2FCB-425C-BA76-00C4CCA9C34F}" name="Table2" displayName="Table2" ref="G6:J13" totalsRowCount="1" headerRowDxfId="52" dataDxfId="53" tableBorderDxfId="57">
   <autoFilter ref="G6:J12" xr:uid="{5A9DE322-2FCB-425C-BA76-00C4CCA9C34F}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{91692FC3-7774-486D-9835-C29BF2D39E5D}" name="Salah " totalsRowLabel="Total" dataDxfId="51" totalsRowDxfId="46"/>
-    <tableColumn id="2" xr3:uid="{0007DC10-F197-4A60-9198-3B136E751393}" name="Nariman " totalsRowFunction="average" dataDxfId="50" totalsRowDxfId="45"/>
-    <tableColumn id="3" xr3:uid="{60A40171-D8F4-4C51-B0D8-419DA8B3324B}" name="Smmar " totalsRowFunction="average" dataDxfId="49" totalsRowDxfId="44"/>
-    <tableColumn id="4" xr3:uid="{F85912A3-6548-467C-8676-2B74640FB6C0}" name="Malak" totalsRowFunction="sum" dataDxfId="42" totalsRowDxfId="43">
+    <tableColumn id="1" xr3:uid="{91692FC3-7774-486D-9835-C29BF2D39E5D}" name="Salah " totalsRowLabel="Total" dataDxfId="56" totalsRowDxfId="51"/>
+    <tableColumn id="2" xr3:uid="{0007DC10-F197-4A60-9198-3B136E751393}" name="Nariman " totalsRowFunction="average" dataDxfId="55" totalsRowDxfId="50"/>
+    <tableColumn id="3" xr3:uid="{60A40171-D8F4-4C51-B0D8-419DA8B3324B}" name="Smmar " totalsRowFunction="average" dataDxfId="54" totalsRowDxfId="49"/>
+    <tableColumn id="4" xr3:uid="{F85912A3-6548-467C-8676-2B74640FB6C0}" name="Malak" totalsRowFunction="sum" dataDxfId="47" totalsRowDxfId="48">
       <calculatedColumnFormula>Table2[[#This Row],[Smmar ]]*Table2[[#This Row],[Nariman ]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1760,76 +1806,91 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{88D28C67-B782-45DE-AC4F-5AE9B1475980}" name="SalesTable" displayName="SalesTable" ref="A1:L101" totalsRowShown="0" headerRowDxfId="34" dataDxfId="33">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{88D28C67-B782-45DE-AC4F-5AE9B1475980}" name="SalesTable" displayName="SalesTable" ref="A1:L101" totalsRowShown="0" headerRowDxfId="39" dataDxfId="38">
   <autoFilter ref="A1:L101" xr:uid="{88D28C67-B782-45DE-AC4F-5AE9B1475980}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{3DAB8B5E-FE74-4509-8E4B-1FBC5C3B0A21}" name="OrderID" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{4E9E9656-0DDA-4C4D-88D7-EAEA6222D00B}" name="Date" dataDxfId="2"/>
-    <tableColumn id="12" xr3:uid="{E6F22816-621B-44C4-92AD-641A35A05678}" name="OrderYear" dataDxfId="1">
+    <tableColumn id="1" xr3:uid="{3DAB8B5E-FE74-4509-8E4B-1FBC5C3B0A21}" name="OrderID" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{4E9E9656-0DDA-4C4D-88D7-EAEA6222D00B}" name="Date" dataDxfId="9"/>
+    <tableColumn id="12" xr3:uid="{E6F22816-621B-44C4-92AD-641A35A05678}" name="OrderYear" dataDxfId="8">
       <calculatedColumnFormula>YEAR(SalesTable[[#This Row],[Date]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{97259138-0FE7-47E5-B631-C8522A70C796}" name="Product" dataDxfId="41"/>
-    <tableColumn id="4" xr3:uid="{1C52AA7A-C71A-45C8-874F-7F1AA567A8CE}" name="Category" dataDxfId="40"/>
-    <tableColumn id="5" xr3:uid="{822E7FC9-678A-4D73-848C-339D14AF94DB}" name="Quantity" dataDxfId="39"/>
-    <tableColumn id="6" xr3:uid="{3C802C12-30D9-4AAA-BC4B-93FC075E0D0D}" name="UnitPrice" dataDxfId="38"/>
-    <tableColumn id="7" xr3:uid="{2EA59F4D-2E9B-4774-83EB-26C335C7DDC6}" name="TotalPrice" dataDxfId="4">
+    <tableColumn id="3" xr3:uid="{97259138-0FE7-47E5-B631-C8522A70C796}" name="Product" dataDxfId="46"/>
+    <tableColumn id="4" xr3:uid="{1C52AA7A-C71A-45C8-874F-7F1AA567A8CE}" name="Category" dataDxfId="45"/>
+    <tableColumn id="5" xr3:uid="{822E7FC9-678A-4D73-848C-339D14AF94DB}" name="Quantity" dataDxfId="44"/>
+    <tableColumn id="6" xr3:uid="{3C802C12-30D9-4AAA-BC4B-93FC075E0D0D}" name="UnitPrice" dataDxfId="43"/>
+    <tableColumn id="7" xr3:uid="{2EA59F4D-2E9B-4774-83EB-26C335C7DDC6}" name="TotalPrice" dataDxfId="11">
       <calculatedColumnFormula>SalesTable[[#This Row],[Quantity]] * SalesTable[[#This Row],[UnitPrice]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{F18B64DF-2AC7-4F69-8B40-A5C2AFFB81E6}" name="CustomerName" dataDxfId="37"/>
-    <tableColumn id="9" xr3:uid="{BE58DA0E-B3AB-43A7-9580-C437394503B1}" name="Email" dataDxfId="36"/>
-    <tableColumn id="13" xr3:uid="{5ADB20C6-E6DF-4BA2-98C4-FFF66329719E}" name="EmailDomain" dataDxfId="0">
+    <tableColumn id="8" xr3:uid="{F18B64DF-2AC7-4F69-8B40-A5C2AFFB81E6}" name="CustomerName" dataDxfId="42"/>
+    <tableColumn id="9" xr3:uid="{BE58DA0E-B3AB-43A7-9580-C437394503B1}" name="Email" dataDxfId="41"/>
+    <tableColumn id="13" xr3:uid="{5ADB20C6-E6DF-4BA2-98C4-FFF66329719E}" name="EmailDomain" dataDxfId="7">
       <calculatedColumnFormula>RIGHT(SalesTable[[#This Row],[Email]], LEN(SalesTable[[#This Row],[Email]]) - FIND("@", SalesTable[[#This Row],[Email]]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{8C3FECA1-992B-400A-9BFF-4F05D3B3E036}" name="Governorate" dataDxfId="35"/>
+    <tableColumn id="10" xr3:uid="{8C3FECA1-992B-400A-9BFF-4F05D3B3E036}" name="Governorate" dataDxfId="40"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{40BF6DF7-3482-4724-9F80-970688912B23}" name="EmployeeTable" displayName="EmployeeTable" ref="A1:I31" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
-  <autoFilter ref="A1:I31" xr:uid="{40BF6DF7-3482-4724-9F80-970688912B23}"/>
-  <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{FF9CF4CE-1FF1-481A-B35E-24E145540DC9}" name="EmployeeID" dataDxfId="32"/>
-    <tableColumn id="2" xr3:uid="{C2708FC9-D605-4B6D-9A78-597CECC1DD7F}" name="FirstName" dataDxfId="31"/>
-    <tableColumn id="3" xr3:uid="{02D02C17-03BD-4199-A3EB-CA2EA74D5867}" name="LastName" dataDxfId="30"/>
-    <tableColumn id="4" xr3:uid="{589B8884-13AF-4D4E-9B97-4D04CB92C587}" name="DateOfBirth" dataDxfId="29"/>
-    <tableColumn id="5" xr3:uid="{754D21C4-7100-4E59-9A80-318BAF48D913}" name="HireDate" dataDxfId="28"/>
-    <tableColumn id="6" xr3:uid="{6875B9AF-01D6-4842-A474-3EAF375EB943}" name="Department" dataDxfId="27"/>
-    <tableColumn id="7" xr3:uid="{8AEC3693-C4F7-49FB-87B4-F0242C6B29B2}" name="Salary" dataDxfId="26"/>
-    <tableColumn id="8" xr3:uid="{A2EA4226-8F5C-4EFA-81DA-5C37336A8F07}" name="PerformanceRating" dataDxfId="25"/>
-    <tableColumn id="9" xr3:uid="{3CED9966-9476-48A6-A0A5-E42DEC0AAA86}" name="Status" dataDxfId="24"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{40BF6DF7-3482-4724-9F80-970688912B23}" name="EmployeeTable" displayName="EmployeeTable" ref="A1:J31" totalsRowShown="0" headerRowDxfId="28" dataDxfId="27">
+  <autoFilter ref="A1:J31" xr:uid="{40BF6DF7-3482-4724-9F80-970688912B23}"/>
+  <tableColumns count="10">
+    <tableColumn id="1" xr3:uid="{FF9CF4CE-1FF1-481A-B35E-24E145540DC9}" name="EmployeeID" dataDxfId="37"/>
+    <tableColumn id="2" xr3:uid="{C2708FC9-D605-4B6D-9A78-597CECC1DD7F}" name="FirstName" dataDxfId="36"/>
+    <tableColumn id="3" xr3:uid="{02D02C17-03BD-4199-A3EB-CA2EA74D5867}" name="LastName" dataDxfId="35"/>
+    <tableColumn id="4" xr3:uid="{589B8884-13AF-4D4E-9B97-4D04CB92C587}" name="DateOfBirth" dataDxfId="34"/>
+    <tableColumn id="5" xr3:uid="{754D21C4-7100-4E59-9A80-318BAF48D913}" name="HireDate" dataDxfId="33"/>
+    <tableColumn id="6" xr3:uid="{6875B9AF-01D6-4842-A474-3EAF375EB943}" name="Department" dataDxfId="32"/>
+    <tableColumn id="10" xr3:uid="{94533672-6467-4E57-BBBF-D9F8F287EE25}" name="DeptHead" dataDxfId="0">
+      <calculatedColumnFormula>_xlfn.XLOOKUP(EmployeeTable[[#This Row],[Department]], Dept_Heads!$A$1:$F$1, Dept_Heads!$A$2:$F$2, "Unassigned")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="7" xr3:uid="{8AEC3693-C4F7-49FB-87B4-F0242C6B29B2}" name="Salary" dataDxfId="31"/>
+    <tableColumn id="8" xr3:uid="{A2EA4226-8F5C-4EFA-81DA-5C37336A8F07}" name="PerformanceRating" dataDxfId="30"/>
+    <tableColumn id="9" xr3:uid="{3CED9966-9476-48A6-A0A5-E42DEC0AAA86}" name="Status" dataDxfId="29"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{B23C9407-1286-4AB5-8DB1-482382F5FEC0}" name="Table8" displayName="Table8" ref="A1:G2" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{B23C9407-1286-4AB5-8DB1-482382F5FEC0}" name="Table8" displayName="Table8" ref="A1:G2" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
   <autoFilter ref="A1:G2" xr:uid="{B23C9407-1286-4AB5-8DB1-482382F5FEC0}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{FCC9D360-8BB3-4547-9B9A-9833EA8115B8}" name="Dept Name" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{2E6A9BC2-0BC6-40B5-80A0-548D1F1EC600}" name="Sales" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{0F027AAA-5F25-41B4-90FD-6D6A6A00E13F}" name="Marketing" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{79038174-9ECB-4730-9E78-CF576BDC90E1}" name="HR" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{57ACCD93-CA87-4B6D-BC2D-7CC7B41FAFC3}" name="IT" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{319C99A9-7FD5-484A-B145-258FAC4FFD29}" name="Finance" dataDxfId="16"/>
-    <tableColumn id="7" xr3:uid="{9351911E-6AA6-4FE2-9820-0F3E7C06C611}" name="Operations" dataDxfId="15"/>
+    <tableColumn id="1" xr3:uid="{FCC9D360-8BB3-4547-9B9A-9833EA8115B8}" name="Dept Name" dataDxfId="26"/>
+    <tableColumn id="2" xr3:uid="{2E6A9BC2-0BC6-40B5-80A0-548D1F1EC600}" name="Sales" dataDxfId="25"/>
+    <tableColumn id="3" xr3:uid="{0F027AAA-5F25-41B4-90FD-6D6A6A00E13F}" name="Marketing" dataDxfId="24"/>
+    <tableColumn id="4" xr3:uid="{79038174-9ECB-4730-9E78-CF576BDC90E1}" name="HR" dataDxfId="23"/>
+    <tableColumn id="5" xr3:uid="{57ACCD93-CA87-4B6D-BC2D-7CC7B41FAFC3}" name="IT" dataDxfId="22"/>
+    <tableColumn id="6" xr3:uid="{319C99A9-7FD5-484A-B145-258FAC4FFD29}" name="Finance" dataDxfId="21"/>
+    <tableColumn id="7" xr3:uid="{9351911E-6AA6-4FE2-9820-0F3E7C06C611}" name="Operations" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{F1D4DEBF-ED57-432F-98A1-ABE9C74E98D7}" name="InventoryTable" displayName="InventoryTable" ref="A1:F52" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
-  <autoFilter ref="A1:F52" xr:uid="{F1D4DEBF-ED57-432F-98A1-ABE9C74E98D7}"/>
-  <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{4B96CD59-37B9-4B41-96D5-DC2F0623D50D}" name="ProductID" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{00738CEB-1827-4D55-A9CE-A4FE252CEF80}" name="ProductName" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{F0AF144B-2612-43A6-9872-8184137AECF0}" name="CurrentStock" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{1921485A-475A-473D-B495-6BFE4A5C0D23}" name="ReorderLevel" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{9A779D84-3E34-4C6F-BC14-5E8FCEA4ACEA}" name="CostPerUnit" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{D3B9E48E-EA6D-4207-9D7E-39A82D741673}" name="SellingPrice" dataDxfId="7"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{F1D4DEBF-ED57-432F-98A1-ABE9C74E98D7}" name="InventoryTable" displayName="InventoryTable" ref="A1:J52" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
+  <autoFilter ref="A1:J52" xr:uid="{F1D4DEBF-ED57-432F-98A1-ABE9C74E98D7}"/>
+  <tableColumns count="10">
+    <tableColumn id="1" xr3:uid="{4B96CD59-37B9-4B41-96D5-DC2F0623D50D}" name="ProductID" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{00738CEB-1827-4D55-A9CE-A4FE252CEF80}" name="ProductName" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{F0AF144B-2612-43A6-9872-8184137AECF0}" name="CurrentStock" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{1921485A-475A-473D-B495-6BFE4A5C0D23}" name="ReorderLevel" dataDxfId="14"/>
+    <tableColumn id="5" xr3:uid="{9A779D84-3E34-4C6F-BC14-5E8FCEA4ACEA}" name="CostPerUnit" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{D3B9E48E-EA6D-4207-9D7E-39A82D741673}" name="SellingPrice" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{D22ABFB5-A424-4FD1-8645-3306FE6BADEB}" name="InventoryValuation" dataDxfId="4">
+      <calculatedColumnFormula>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="8" xr3:uid="{9FFD8FDF-2F6F-44EB-94A0-3FEA8B0AB89C}" name="GrossMarginEGP" dataDxfId="3">
+      <calculatedColumnFormula>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="9" xr3:uid="{C3160D59-8734-48A1-B1AD-45FAA97E162C}" name="MarkupPercentage" dataDxfId="2">
+      <calculatedColumnFormula>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="10" xr3:uid="{2C6056C7-B8DE-4071-92C9-33BCB35B07DB}" name="ReorderAlert" dataDxfId="1">
+      <calculatedColumnFormula>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6527,7 +6588,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.5546875" bestFit="1" customWidth="1"/>
@@ -6535,12 +6596,13 @@
     <col min="3" max="3" width="13.77734375" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="17" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.5546875" customWidth="1"/>
+    <col min="8" max="8" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="16" t="s">
         <v>185</v>
       </c>
@@ -6560,16 +6622,19 @@
         <v>190</v>
       </c>
       <c r="G1" s="16" t="s">
+        <v>359</v>
+      </c>
+      <c r="H1" s="16" t="s">
         <v>191</v>
       </c>
-      <c r="H1" s="16" t="s">
+      <c r="I1" s="16" t="s">
         <v>192</v>
       </c>
-      <c r="I1" s="16" t="s">
+      <c r="J1" s="16" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="16" t="s">
         <v>194</v>
       </c>
@@ -6588,17 +6653,21 @@
       <c r="F2" s="16" t="s">
         <v>197</v>
       </c>
-      <c r="G2" s="16">
+      <c r="G2" s="16" t="str">
+        <f>_xlfn.XLOOKUP(EmployeeTable[[#This Row],[Department]], Dept_Heads!$A$1:$F$1, Dept_Heads!$A$2:$F$2, "Unassigned")</f>
+        <v>Fatima Nour</v>
+      </c>
+      <c r="H2" s="16">
         <v>23447</v>
       </c>
-      <c r="H2" s="16">
+      <c r="I2" s="16">
         <v>2</v>
       </c>
-      <c r="I2" s="16" t="s">
+      <c r="J2" s="16" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="16" t="s">
         <v>199</v>
       </c>
@@ -6617,17 +6686,21 @@
       <c r="F3" s="16" t="s">
         <v>197</v>
       </c>
-      <c r="G3" s="16">
+      <c r="G3" s="16" t="str">
+        <f>_xlfn.XLOOKUP(EmployeeTable[[#This Row],[Department]], Dept_Heads!$A$1:$F$1, Dept_Heads!$A$2:$F$2, "Unassigned")</f>
+        <v>Fatima Nour</v>
+      </c>
+      <c r="H3" s="16">
         <v>8983</v>
       </c>
-      <c r="H3" s="16">
+      <c r="I3" s="16">
         <v>3</v>
       </c>
-      <c r="I3" s="16" t="s">
+      <c r="J3" s="16" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="16" t="s">
         <v>203</v>
       </c>
@@ -6646,17 +6719,21 @@
       <c r="F4" s="16" t="s">
         <v>205</v>
       </c>
-      <c r="G4" s="16">
+      <c r="G4" s="16" t="str">
+        <f>_xlfn.XLOOKUP(EmployeeTable[[#This Row],[Department]], Dept_Heads!$A$1:$F$1, Dept_Heads!$A$2:$F$2, "Unassigned")</f>
+        <v>Unassigned</v>
+      </c>
+      <c r="H4" s="16">
         <v>10949</v>
       </c>
-      <c r="H4" s="16">
+      <c r="I4" s="16">
         <v>3</v>
       </c>
-      <c r="I4" s="16" t="s">
+      <c r="J4" s="16" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="16" t="s">
         <v>206</v>
       </c>
@@ -6675,17 +6752,21 @@
       <c r="F5" s="16" t="s">
         <v>205</v>
       </c>
-      <c r="G5" s="16">
+      <c r="G5" s="16" t="str">
+        <f>_xlfn.XLOOKUP(EmployeeTable[[#This Row],[Department]], Dept_Heads!$A$1:$F$1, Dept_Heads!$A$2:$F$2, "Unassigned")</f>
+        <v>Unassigned</v>
+      </c>
+      <c r="H5" s="16">
         <v>18312</v>
       </c>
-      <c r="H5" s="16">
+      <c r="I5" s="16">
         <v>2</v>
       </c>
-      <c r="I5" s="16" t="s">
+      <c r="J5" s="16" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="16" t="s">
         <v>210</v>
       </c>
@@ -6704,17 +6785,21 @@
       <c r="F6" s="16" t="s">
         <v>213</v>
       </c>
-      <c r="G6" s="16">
+      <c r="G6" s="16" t="str">
+        <f>_xlfn.XLOOKUP(EmployeeTable[[#This Row],[Department]], Dept_Heads!$A$1:$F$1, Dept_Heads!$A$2:$F$2, "Unassigned")</f>
+        <v>Yasmin Hassan</v>
+      </c>
+      <c r="H6" s="16">
         <v>19671</v>
       </c>
-      <c r="H6" s="16">
+      <c r="I6" s="16">
         <v>3</v>
       </c>
-      <c r="I6" s="16" t="s">
+      <c r="J6" s="16" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="16" t="s">
         <v>214</v>
       </c>
@@ -6733,17 +6818,21 @@
       <c r="F7" s="16" t="s">
         <v>216</v>
       </c>
-      <c r="G7" s="16">
+      <c r="G7" s="16" t="str">
+        <f>_xlfn.XLOOKUP(EmployeeTable[[#This Row],[Department]], Dept_Heads!$A$1:$F$1, Dept_Heads!$A$2:$F$2, "Unassigned")</f>
+        <v>Omar Farouk</v>
+      </c>
+      <c r="H7" s="16">
         <v>9345</v>
       </c>
-      <c r="H7" s="16">
+      <c r="I7" s="16">
         <v>5</v>
       </c>
-      <c r="I7" s="16" t="s">
+      <c r="J7" s="16" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="16" t="s">
         <v>217</v>
       </c>
@@ -6762,17 +6851,21 @@
       <c r="F8" s="16" t="s">
         <v>205</v>
       </c>
-      <c r="G8" s="16">
+      <c r="G8" s="16" t="str">
+        <f>_xlfn.XLOOKUP(EmployeeTable[[#This Row],[Department]], Dept_Heads!$A$1:$F$1, Dept_Heads!$A$2:$F$2, "Unassigned")</f>
+        <v>Unassigned</v>
+      </c>
+      <c r="H8" s="16">
         <v>23667</v>
       </c>
-      <c r="H8" s="16">
+      <c r="I8" s="16">
         <v>5</v>
       </c>
-      <c r="I8" s="16" t="s">
+      <c r="J8" s="16" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="16" t="s">
         <v>220</v>
       </c>
@@ -6791,17 +6884,21 @@
       <c r="F9" s="16" t="s">
         <v>222</v>
       </c>
-      <c r="G9" s="16">
+      <c r="G9" s="16" t="str">
+        <f>_xlfn.XLOOKUP(EmployeeTable[[#This Row],[Department]], Dept_Heads!$A$1:$F$1, Dept_Heads!$A$2:$F$2, "Unassigned")</f>
+        <v>Mohamed Samir</v>
+      </c>
+      <c r="H9" s="16">
         <v>9615</v>
       </c>
-      <c r="H9" s="16">
+      <c r="I9" s="16">
         <v>3</v>
       </c>
-      <c r="I9" s="16" t="s">
+      <c r="J9" s="16" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="16" t="s">
         <v>223</v>
       </c>
@@ -6820,17 +6917,21 @@
       <c r="F10" s="16" t="s">
         <v>216</v>
       </c>
-      <c r="G10" s="16">
+      <c r="G10" s="16" t="str">
+        <f>_xlfn.XLOOKUP(EmployeeTable[[#This Row],[Department]], Dept_Heads!$A$1:$F$1, Dept_Heads!$A$2:$F$2, "Unassigned")</f>
+        <v>Omar Farouk</v>
+      </c>
+      <c r="H10" s="16">
         <v>10066</v>
       </c>
-      <c r="H10" s="16">
+      <c r="I10" s="16">
         <v>3</v>
       </c>
-      <c r="I10" s="16" t="s">
+      <c r="J10" s="16" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="16" t="s">
         <v>226</v>
       </c>
@@ -6849,17 +6950,21 @@
       <c r="F11" s="16" t="s">
         <v>205</v>
       </c>
-      <c r="G11" s="16">
+      <c r="G11" s="16" t="str">
+        <f>_xlfn.XLOOKUP(EmployeeTable[[#This Row],[Department]], Dept_Heads!$A$1:$F$1, Dept_Heads!$A$2:$F$2, "Unassigned")</f>
+        <v>Unassigned</v>
+      </c>
+      <c r="H11" s="16">
         <v>20787</v>
       </c>
-      <c r="H11" s="16">
+      <c r="I11" s="16">
         <v>1</v>
       </c>
-      <c r="I11" s="16" t="s">
+      <c r="J11" s="16" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="16" t="s">
         <v>228</v>
       </c>
@@ -6878,17 +6983,21 @@
       <c r="F12" s="16" t="s">
         <v>205</v>
       </c>
-      <c r="G12" s="16">
+      <c r="G12" s="16" t="str">
+        <f>_xlfn.XLOOKUP(EmployeeTable[[#This Row],[Department]], Dept_Heads!$A$1:$F$1, Dept_Heads!$A$2:$F$2, "Unassigned")</f>
+        <v>Unassigned</v>
+      </c>
+      <c r="H12" s="16">
         <v>10631</v>
       </c>
-      <c r="H12" s="16">
+      <c r="I12" s="16">
         <v>4</v>
       </c>
-      <c r="I12" s="16" t="s">
+      <c r="J12" s="16" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="16" t="s">
         <v>230</v>
       </c>
@@ -6907,17 +7016,21 @@
       <c r="F13" s="16" t="s">
         <v>216</v>
       </c>
-      <c r="G13" s="16">
+      <c r="G13" s="16" t="str">
+        <f>_xlfn.XLOOKUP(EmployeeTable[[#This Row],[Department]], Dept_Heads!$A$1:$F$1, Dept_Heads!$A$2:$F$2, "Unassigned")</f>
+        <v>Omar Farouk</v>
+      </c>
+      <c r="H13" s="16">
         <v>20190</v>
       </c>
-      <c r="H13" s="16">
+      <c r="I13" s="16">
         <v>4</v>
       </c>
-      <c r="I13" s="16" t="s">
+      <c r="J13" s="16" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="16" t="s">
         <v>233</v>
       </c>
@@ -6936,17 +7049,21 @@
       <c r="F14" s="16" t="s">
         <v>222</v>
       </c>
-      <c r="G14" s="16">
+      <c r="G14" s="16" t="str">
+        <f>_xlfn.XLOOKUP(EmployeeTable[[#This Row],[Department]], Dept_Heads!$A$1:$F$1, Dept_Heads!$A$2:$F$2, "Unassigned")</f>
+        <v>Mohamed Samir</v>
+      </c>
+      <c r="H14" s="16">
         <v>24565</v>
       </c>
-      <c r="H14" s="16">
+      <c r="I14" s="16">
         <v>2</v>
       </c>
-      <c r="I14" s="16" t="s">
+      <c r="J14" s="16" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="16" t="s">
         <v>235</v>
       </c>
@@ -6965,17 +7082,21 @@
       <c r="F15" s="16" t="s">
         <v>197</v>
       </c>
-      <c r="G15" s="16">
+      <c r="G15" s="16" t="str">
+        <f>_xlfn.XLOOKUP(EmployeeTable[[#This Row],[Department]], Dept_Heads!$A$1:$F$1, Dept_Heads!$A$2:$F$2, "Unassigned")</f>
+        <v>Fatima Nour</v>
+      </c>
+      <c r="H15" s="16">
         <v>17746</v>
       </c>
-      <c r="H15" s="16">
+      <c r="I15" s="16">
         <v>2</v>
       </c>
-      <c r="I15" s="16" t="s">
+      <c r="J15" s="16" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="16" t="s">
         <v>238</v>
       </c>
@@ -6994,17 +7115,21 @@
       <c r="F16" s="16" t="s">
         <v>239</v>
       </c>
-      <c r="G16" s="16">
+      <c r="G16" s="16" t="str">
+        <f>_xlfn.XLOOKUP(EmployeeTable[[#This Row],[Department]], Dept_Heads!$A$1:$F$1, Dept_Heads!$A$2:$F$2, "Unassigned")</f>
+        <v>Ahmed El-Masry</v>
+      </c>
+      <c r="H16" s="16">
         <v>14806</v>
       </c>
-      <c r="H16" s="16">
+      <c r="I16" s="16">
         <v>1</v>
       </c>
-      <c r="I16" s="16" t="s">
+      <c r="J16" s="16" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="16" t="s">
         <v>240</v>
       </c>
@@ -7023,17 +7148,21 @@
       <c r="F17" s="16" t="s">
         <v>213</v>
       </c>
-      <c r="G17" s="16">
+      <c r="G17" s="16" t="str">
+        <f>_xlfn.XLOOKUP(EmployeeTable[[#This Row],[Department]], Dept_Heads!$A$1:$F$1, Dept_Heads!$A$2:$F$2, "Unassigned")</f>
+        <v>Yasmin Hassan</v>
+      </c>
+      <c r="H17" s="16">
         <v>20180</v>
       </c>
-      <c r="H17" s="16">
+      <c r="I17" s="16">
         <v>2</v>
       </c>
-      <c r="I17" s="16" t="s">
+      <c r="J17" s="16" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="16" t="s">
         <v>241</v>
       </c>
@@ -7052,17 +7181,21 @@
       <c r="F18" s="16" t="s">
         <v>222</v>
       </c>
-      <c r="G18" s="16">
+      <c r="G18" s="16" t="str">
+        <f>_xlfn.XLOOKUP(EmployeeTable[[#This Row],[Department]], Dept_Heads!$A$1:$F$1, Dept_Heads!$A$2:$F$2, "Unassigned")</f>
+        <v>Mohamed Samir</v>
+      </c>
+      <c r="H18" s="16">
         <v>12728</v>
       </c>
-      <c r="H18" s="16">
+      <c r="I18" s="16">
         <v>5</v>
       </c>
-      <c r="I18" s="16" t="s">
+      <c r="J18" s="16" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="16" t="s">
         <v>242</v>
       </c>
@@ -7081,17 +7214,21 @@
       <c r="F19" s="16" t="s">
         <v>216</v>
       </c>
-      <c r="G19" s="16">
+      <c r="G19" s="16" t="str">
+        <f>_xlfn.XLOOKUP(EmployeeTable[[#This Row],[Department]], Dept_Heads!$A$1:$F$1, Dept_Heads!$A$2:$F$2, "Unassigned")</f>
+        <v>Omar Farouk</v>
+      </c>
+      <c r="H19" s="16">
         <v>16783</v>
       </c>
-      <c r="H19" s="16">
+      <c r="I19" s="16">
         <v>2</v>
       </c>
-      <c r="I19" s="16" t="s">
+      <c r="J19" s="16" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="16" t="s">
         <v>243</v>
       </c>
@@ -7110,17 +7247,21 @@
       <c r="F20" s="16" t="s">
         <v>197</v>
       </c>
-      <c r="G20" s="16">
+      <c r="G20" s="16" t="str">
+        <f>_xlfn.XLOOKUP(EmployeeTable[[#This Row],[Department]], Dept_Heads!$A$1:$F$1, Dept_Heads!$A$2:$F$2, "Unassigned")</f>
+        <v>Fatima Nour</v>
+      </c>
+      <c r="H20" s="16">
         <v>9944</v>
       </c>
-      <c r="H20" s="16">
+      <c r="I20" s="16">
         <v>1</v>
       </c>
-      <c r="I20" s="16" t="s">
+      <c r="J20" s="16" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="16" t="s">
         <v>245</v>
       </c>
@@ -7139,17 +7280,21 @@
       <c r="F21" s="16" t="s">
         <v>197</v>
       </c>
-      <c r="G21" s="16">
+      <c r="G21" s="16" t="str">
+        <f>_xlfn.XLOOKUP(EmployeeTable[[#This Row],[Department]], Dept_Heads!$A$1:$F$1, Dept_Heads!$A$2:$F$2, "Unassigned")</f>
+        <v>Fatima Nour</v>
+      </c>
+      <c r="H21" s="16">
         <v>14882</v>
       </c>
-      <c r="H21" s="16">
+      <c r="I21" s="16">
         <v>4</v>
       </c>
-      <c r="I21" s="16" t="s">
+      <c r="J21" s="16" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" s="16" t="s">
         <v>248</v>
       </c>
@@ -7168,17 +7313,21 @@
       <c r="F22" s="16" t="s">
         <v>197</v>
       </c>
-      <c r="G22" s="16">
+      <c r="G22" s="16" t="str">
+        <f>_xlfn.XLOOKUP(EmployeeTable[[#This Row],[Department]], Dept_Heads!$A$1:$F$1, Dept_Heads!$A$2:$F$2, "Unassigned")</f>
+        <v>Fatima Nour</v>
+      </c>
+      <c r="H22" s="16">
         <v>13524</v>
       </c>
-      <c r="H22" s="16">
+      <c r="I22" s="16">
         <v>2</v>
       </c>
-      <c r="I22" s="16" t="s">
+      <c r="J22" s="16" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" s="16" t="s">
         <v>249</v>
       </c>
@@ -7197,17 +7346,21 @@
       <c r="F23" s="16" t="s">
         <v>205</v>
       </c>
-      <c r="G23" s="16">
+      <c r="G23" s="16" t="str">
+        <f>_xlfn.XLOOKUP(EmployeeTable[[#This Row],[Department]], Dept_Heads!$A$1:$F$1, Dept_Heads!$A$2:$F$2, "Unassigned")</f>
+        <v>Unassigned</v>
+      </c>
+      <c r="H23" s="16">
         <v>23405</v>
       </c>
-      <c r="H23" s="16">
+      <c r="I23" s="16">
         <v>4</v>
       </c>
-      <c r="I23" s="16" t="s">
+      <c r="J23" s="16" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" s="16" t="s">
         <v>251</v>
       </c>
@@ -7226,17 +7379,21 @@
       <c r="F24" s="16" t="s">
         <v>205</v>
       </c>
-      <c r="G24" s="16">
+      <c r="G24" s="16" t="str">
+        <f>_xlfn.XLOOKUP(EmployeeTable[[#This Row],[Department]], Dept_Heads!$A$1:$F$1, Dept_Heads!$A$2:$F$2, "Unassigned")</f>
+        <v>Unassigned</v>
+      </c>
+      <c r="H24" s="16">
         <v>23580</v>
       </c>
-      <c r="H24" s="16">
+      <c r="I24" s="16">
         <v>3</v>
       </c>
-      <c r="I24" s="16" t="s">
+      <c r="J24" s="16" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" s="16" t="s">
         <v>252</v>
       </c>
@@ -7255,17 +7412,21 @@
       <c r="F25" s="16" t="s">
         <v>239</v>
       </c>
-      <c r="G25" s="16">
+      <c r="G25" s="16" t="str">
+        <f>_xlfn.XLOOKUP(EmployeeTable[[#This Row],[Department]], Dept_Heads!$A$1:$F$1, Dept_Heads!$A$2:$F$2, "Unassigned")</f>
+        <v>Ahmed El-Masry</v>
+      </c>
+      <c r="H25" s="16">
         <v>24424</v>
       </c>
-      <c r="H25" s="16">
+      <c r="I25" s="16">
         <v>3</v>
       </c>
-      <c r="I25" s="16" t="s">
+      <c r="J25" s="16" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="16" t="s">
         <v>253</v>
       </c>
@@ -7284,17 +7445,21 @@
       <c r="F26" s="16" t="s">
         <v>213</v>
       </c>
-      <c r="G26" s="16">
+      <c r="G26" s="16" t="str">
+        <f>_xlfn.XLOOKUP(EmployeeTable[[#This Row],[Department]], Dept_Heads!$A$1:$F$1, Dept_Heads!$A$2:$F$2, "Unassigned")</f>
+        <v>Yasmin Hassan</v>
+      </c>
+      <c r="H26" s="16">
         <v>14822</v>
       </c>
-      <c r="H26" s="16">
+      <c r="I26" s="16">
         <v>4</v>
       </c>
-      <c r="I26" s="16" t="s">
+      <c r="J26" s="16" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="16" t="s">
         <v>254</v>
       </c>
@@ -7313,17 +7478,21 @@
       <c r="F27" s="16" t="s">
         <v>239</v>
       </c>
-      <c r="G27" s="16">
+      <c r="G27" s="16" t="str">
+        <f>_xlfn.XLOOKUP(EmployeeTable[[#This Row],[Department]], Dept_Heads!$A$1:$F$1, Dept_Heads!$A$2:$F$2, "Unassigned")</f>
+        <v>Ahmed El-Masry</v>
+      </c>
+      <c r="H27" s="16">
         <v>13177</v>
       </c>
-      <c r="H27" s="16">
+      <c r="I27" s="16">
         <v>3</v>
       </c>
-      <c r="I27" s="16" t="s">
+      <c r="J27" s="16" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="16" t="s">
         <v>256</v>
       </c>
@@ -7342,17 +7511,21 @@
       <c r="F28" s="16" t="s">
         <v>197</v>
       </c>
-      <c r="G28" s="16">
+      <c r="G28" s="16" t="str">
+        <f>_xlfn.XLOOKUP(EmployeeTable[[#This Row],[Department]], Dept_Heads!$A$1:$F$1, Dept_Heads!$A$2:$F$2, "Unassigned")</f>
+        <v>Fatima Nour</v>
+      </c>
+      <c r="H28" s="16">
         <v>8083</v>
       </c>
-      <c r="H28" s="16">
+      <c r="I28" s="16">
         <v>2</v>
       </c>
-      <c r="I28" s="16" t="s">
+      <c r="J28" s="16" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" s="16" t="s">
         <v>258</v>
       </c>
@@ -7371,17 +7544,21 @@
       <c r="F29" s="16" t="s">
         <v>197</v>
       </c>
-      <c r="G29" s="16">
+      <c r="G29" s="16" t="str">
+        <f>_xlfn.XLOOKUP(EmployeeTable[[#This Row],[Department]], Dept_Heads!$A$1:$F$1, Dept_Heads!$A$2:$F$2, "Unassigned")</f>
+        <v>Fatima Nour</v>
+      </c>
+      <c r="H29" s="16">
         <v>14386</v>
       </c>
-      <c r="H29" s="16">
+      <c r="I29" s="16">
         <v>2</v>
       </c>
-      <c r="I29" s="16" t="s">
+      <c r="J29" s="16" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="16" t="s">
         <v>260</v>
       </c>
@@ -7400,17 +7577,21 @@
       <c r="F30" s="16" t="s">
         <v>239</v>
       </c>
-      <c r="G30" s="16">
+      <c r="G30" s="16" t="str">
+        <f>_xlfn.XLOOKUP(EmployeeTable[[#This Row],[Department]], Dept_Heads!$A$1:$F$1, Dept_Heads!$A$2:$F$2, "Unassigned")</f>
+        <v>Ahmed El-Masry</v>
+      </c>
+      <c r="H30" s="16">
         <v>18139</v>
       </c>
-      <c r="H30" s="16">
+      <c r="I30" s="16">
         <v>4</v>
       </c>
-      <c r="I30" s="16" t="s">
+      <c r="J30" s="16" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" s="16" t="s">
         <v>261</v>
       </c>
@@ -7429,13 +7610,17 @@
       <c r="F31" s="16" t="s">
         <v>197</v>
       </c>
-      <c r="G31" s="16">
+      <c r="G31" s="16" t="str">
+        <f>_xlfn.XLOOKUP(EmployeeTable[[#This Row],[Department]], Dept_Heads!$A$1:$F$1, Dept_Heads!$A$2:$F$2, "Unassigned")</f>
+        <v>Fatima Nour</v>
+      </c>
+      <c r="H31" s="16">
         <v>22117</v>
       </c>
-      <c r="H31" s="16">
+      <c r="I31" s="16">
         <v>4</v>
       </c>
-      <c r="I31" s="16" t="s">
+      <c r="J31" s="16" t="s">
         <v>198</v>
       </c>
     </row>
@@ -7517,17 +7702,21 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:F52"/>
+  <dimension ref="A1:J52"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.44140625" style="23" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15" style="23" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22" style="23" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.44140625" style="23" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.77734375" style="25" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="16" t="s">
         <v>268</v>
       </c>
@@ -7540,14 +7729,26 @@
       <c r="D1" s="16" t="s">
         <v>271</v>
       </c>
-      <c r="E1" s="16" t="s">
+      <c r="E1" s="22" t="s">
         <v>272</v>
       </c>
-      <c r="F1" s="16" t="s">
+      <c r="F1" s="22" t="s">
         <v>273</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G1" s="22" t="s">
+        <v>355</v>
+      </c>
+      <c r="H1" s="22" t="s">
+        <v>356</v>
+      </c>
+      <c r="I1" s="24" t="s">
+        <v>357</v>
+      </c>
+      <c r="J1" s="16" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="16" t="s">
         <v>274</v>
       </c>
@@ -7560,14 +7761,30 @@
       <c r="D2" s="16">
         <v>39</v>
       </c>
-      <c r="E2" s="16">
+      <c r="E2" s="22">
         <v>1157.48</v>
       </c>
-      <c r="F2" s="16">
+      <c r="F2" s="22">
         <v>1364.39</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G2" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>226866.08000000002</v>
+      </c>
+      <c r="H2" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>206.91000000000008</v>
+      </c>
+      <c r="I2" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.17875902823374926</v>
+      </c>
+      <c r="J2" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="16" t="s">
         <v>276</v>
       </c>
@@ -7580,14 +7797,30 @@
       <c r="D3" s="16">
         <v>34</v>
       </c>
-      <c r="E3" s="16">
+      <c r="E3" s="22">
         <v>454.44</v>
       </c>
-      <c r="F3" s="16">
+      <c r="F3" s="22">
         <v>666.38</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G3" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>48170.64</v>
+      </c>
+      <c r="H3" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>211.94</v>
+      </c>
+      <c r="I3" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.46637619927823254</v>
+      </c>
+      <c r="J3" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="16" t="s">
         <v>278</v>
       </c>
@@ -7600,14 +7833,30 @@
       <c r="D4" s="16">
         <v>17</v>
       </c>
-      <c r="E4" s="16">
+      <c r="E4" s="22">
         <v>1200.1400000000001</v>
       </c>
-      <c r="F4" s="16">
+      <c r="F4" s="22">
         <v>1655.78</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G4" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>171620.02000000002</v>
+      </c>
+      <c r="H4" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>455.63999999999987</v>
+      </c>
+      <c r="I4" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.37965570683420252</v>
+      </c>
+      <c r="J4" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="16" t="s">
         <v>280</v>
       </c>
@@ -7620,14 +7869,30 @@
       <c r="D5" s="16">
         <v>35</v>
       </c>
-      <c r="E5" s="16">
+      <c r="E5" s="22">
         <v>1114.1099999999999</v>
       </c>
-      <c r="F5" s="16">
+      <c r="F5" s="22">
         <v>1525.88</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G5" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>33423.299999999996</v>
+      </c>
+      <c r="H5" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>411.77000000000021</v>
+      </c>
+      <c r="I5" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.3695954618484712</v>
+      </c>
+      <c r="J5" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>REORDER REQUIRED</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="16" t="s">
         <v>282</v>
       </c>
@@ -7640,14 +7905,30 @@
       <c r="D6" s="16">
         <v>48</v>
       </c>
-      <c r="E6" s="16">
+      <c r="E6" s="22">
         <v>546.80999999999995</v>
       </c>
-      <c r="F6" s="16">
+      <c r="F6" s="22">
         <v>702.42</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G6" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>91317.26999999999</v>
+      </c>
+      <c r="H6" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>155.61000000000001</v>
+      </c>
+      <c r="I6" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.28457782410709392</v>
+      </c>
+      <c r="J6" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="16" t="s">
         <v>284</v>
       </c>
@@ -7660,14 +7941,30 @@
       <c r="D7" s="16">
         <v>37</v>
       </c>
-      <c r="E7" s="16">
+      <c r="E7" s="22">
         <v>2046.35</v>
       </c>
-      <c r="F7" s="16">
+      <c r="F7" s="22">
         <v>3040.26</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G7" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>284442.64999999997</v>
+      </c>
+      <c r="H7" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>993.91000000000031</v>
+      </c>
+      <c r="I7" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.4856989273584677</v>
+      </c>
+      <c r="J7" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="16" t="s">
         <v>286</v>
       </c>
@@ -7680,14 +7977,30 @@
       <c r="D8" s="16">
         <v>20</v>
       </c>
-      <c r="E8" s="16">
+      <c r="E8" s="22">
         <v>1625.13</v>
       </c>
-      <c r="F8" s="16">
+      <c r="F8" s="22">
         <v>1804.95</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G8" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>92632.41</v>
+      </c>
+      <c r="H8" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>179.81999999999994</v>
+      </c>
+      <c r="I8" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.11064960956969591</v>
+      </c>
+      <c r="J8" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="16" t="s">
         <v>287</v>
       </c>
@@ -7700,14 +8013,30 @@
       <c r="D9" s="16">
         <v>12</v>
       </c>
-      <c r="E9" s="16">
+      <c r="E9" s="22">
         <v>1593.15</v>
       </c>
-      <c r="F9" s="16">
+      <c r="F9" s="22">
         <v>2306.94</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G9" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>133824.6</v>
+      </c>
+      <c r="H9" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>713.79</v>
+      </c>
+      <c r="I9" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.44803690801242818</v>
+      </c>
+      <c r="J9" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="16" t="s">
         <v>288</v>
       </c>
@@ -7720,14 +8049,30 @@
       <c r="D10" s="16">
         <v>34</v>
       </c>
-      <c r="E10" s="16">
+      <c r="E10" s="22">
         <v>317.17</v>
       </c>
-      <c r="F10" s="16">
+      <c r="F10" s="22">
         <v>460.2</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G10" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>62482.490000000005</v>
+      </c>
+      <c r="H10" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>143.02999999999997</v>
+      </c>
+      <c r="I10" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.45095690008512773</v>
+      </c>
+      <c r="J10" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="16" t="s">
         <v>290</v>
       </c>
@@ -7740,14 +8085,30 @@
       <c r="D11" s="16">
         <v>47</v>
       </c>
-      <c r="E11" s="16">
+      <c r="E11" s="22">
         <v>2477.0100000000002</v>
       </c>
-      <c r="F11" s="16">
+      <c r="F11" s="22">
         <v>3630.79</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G11" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>329442.33</v>
+      </c>
+      <c r="H11" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>1153.7799999999997</v>
+      </c>
+      <c r="I11" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.46579545500421865</v>
+      </c>
+      <c r="J11" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="16" t="s">
         <v>292</v>
       </c>
@@ -7760,14 +8121,30 @@
       <c r="D12" s="16">
         <v>26</v>
       </c>
-      <c r="E12" s="16">
+      <c r="E12" s="22">
         <v>951.38</v>
       </c>
-      <c r="F12" s="16">
+      <c r="F12" s="22">
         <v>1047.8399999999999</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G12" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>36152.44</v>
+      </c>
+      <c r="H12" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>96.459999999999923</v>
+      </c>
+      <c r="I12" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.10138956042800976</v>
+      </c>
+      <c r="J12" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="16" t="s">
         <v>294</v>
       </c>
@@ -7780,14 +8157,30 @@
       <c r="D13" s="16">
         <v>13</v>
       </c>
-      <c r="E13" s="16">
+      <c r="E13" s="22">
         <v>1288.1099999999999</v>
       </c>
-      <c r="F13" s="16">
+      <c r="F13" s="22">
         <v>1748.08</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G13" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>256333.88999999998</v>
+      </c>
+      <c r="H13" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>459.97</v>
+      </c>
+      <c r="I13" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.35708906848017641</v>
+      </c>
+      <c r="J13" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="16" t="s">
         <v>296</v>
       </c>
@@ -7800,14 +8193,30 @@
       <c r="D14" s="16">
         <v>43</v>
       </c>
-      <c r="E14" s="16">
+      <c r="E14" s="22">
         <v>1629.29</v>
       </c>
-      <c r="F14" s="16">
+      <c r="F14" s="22">
         <v>2207.94</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G14" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>125455.33</v>
+      </c>
+      <c r="H14" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>578.65000000000009</v>
+      </c>
+      <c r="I14" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.3551546992861922</v>
+      </c>
+      <c r="J14" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="16" t="s">
         <v>297</v>
       </c>
@@ -7820,14 +8229,30 @@
       <c r="D15" s="16">
         <v>47</v>
       </c>
-      <c r="E15" s="16">
+      <c r="E15" s="22">
         <v>2111.65</v>
       </c>
-      <c r="F15" s="16">
+      <c r="F15" s="22">
         <v>3068.95</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G15" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>33786.400000000001</v>
+      </c>
+      <c r="H15" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>957.29999999999973</v>
+      </c>
+      <c r="I15" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.45334217318210862</v>
+      </c>
+      <c r="J15" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>REORDER REQUIRED</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="16" t="s">
         <v>298</v>
       </c>
@@ -7840,14 +8265,30 @@
       <c r="D16" s="16">
         <v>23</v>
       </c>
-      <c r="E16" s="16">
+      <c r="E16" s="22">
         <v>1799.62</v>
       </c>
-      <c r="F16" s="16">
+      <c r="F16" s="22">
         <v>2081.9699999999998</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G16" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>102578.34</v>
+      </c>
+      <c r="H16" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>282.34999999999991</v>
+      </c>
+      <c r="I16" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.15689423322701454</v>
+      </c>
+      <c r="J16" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="16" t="s">
         <v>299</v>
       </c>
@@ -7860,14 +8301,30 @@
       <c r="D17" s="16">
         <v>48</v>
       </c>
-      <c r="E17" s="16">
+      <c r="E17" s="22">
         <v>1187.71</v>
       </c>
-      <c r="F17" s="16">
+      <c r="F17" s="22">
         <v>1342.5</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G17" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>112832.45</v>
+      </c>
+      <c r="H17" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>154.78999999999996</v>
+      </c>
+      <c r="I17" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.13032642648457954</v>
+      </c>
+      <c r="J17" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="16" t="s">
         <v>300</v>
       </c>
@@ -7880,14 +8337,30 @@
       <c r="D18" s="16">
         <v>28</v>
       </c>
-      <c r="E18" s="16">
+      <c r="E18" s="22">
         <v>65.86</v>
       </c>
-      <c r="F18" s="16">
+      <c r="F18" s="22">
         <v>93.02</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G18" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>7903.2</v>
+      </c>
+      <c r="H18" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>27.159999999999997</v>
+      </c>
+      <c r="I18" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.41238991800789548</v>
+      </c>
+      <c r="J18" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="16" t="s">
         <v>302</v>
       </c>
@@ -7900,14 +8373,30 @@
       <c r="D19" s="16">
         <v>26</v>
       </c>
-      <c r="E19" s="16">
+      <c r="E19" s="22">
         <v>1905.31</v>
       </c>
-      <c r="F19" s="16">
+      <c r="F19" s="22">
         <v>2642.42</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G19" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>209584.1</v>
+      </c>
+      <c r="H19" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>737.11000000000013</v>
+      </c>
+      <c r="I19" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.386871427746666</v>
+      </c>
+      <c r="J19" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="16" t="s">
         <v>304</v>
       </c>
@@ -7920,14 +8409,30 @@
       <c r="D20" s="16">
         <v>12</v>
       </c>
-      <c r="E20" s="16">
+      <c r="E20" s="22">
         <v>1615.61</v>
       </c>
-      <c r="F20" s="16">
+      <c r="F20" s="22">
         <v>2039.38</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G20" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>203566.86</v>
+      </c>
+      <c r="H20" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>423.77000000000021</v>
+      </c>
+      <c r="I20" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.26229721281744989</v>
+      </c>
+      <c r="J20" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="16" t="s">
         <v>306</v>
       </c>
@@ -7940,14 +8445,30 @@
       <c r="D21" s="16">
         <v>25</v>
       </c>
-      <c r="E21" s="16">
+      <c r="E21" s="22">
         <v>1606.66</v>
       </c>
-      <c r="F21" s="16">
+      <c r="F21" s="22">
         <v>2051.9299999999998</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G21" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>260278.92</v>
+      </c>
+      <c r="H21" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>445.26999999999975</v>
+      </c>
+      <c r="I21" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.27714015410852311</v>
+      </c>
+      <c r="J21" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" s="16" t="s">
         <v>308</v>
       </c>
@@ -7960,14 +8481,30 @@
       <c r="D22" s="16">
         <v>39</v>
       </c>
-      <c r="E22" s="16">
+      <c r="E22" s="22">
         <v>2098.96</v>
       </c>
-      <c r="F22" s="16">
+      <c r="F22" s="22">
         <v>2706.12</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G22" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>149026.16</v>
+      </c>
+      <c r="H22" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>607.15999999999985</v>
+      </c>
+      <c r="I22" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.28926706559438953</v>
+      </c>
+      <c r="J22" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" s="16" t="s">
         <v>309</v>
       </c>
@@ -7980,14 +8517,30 @@
       <c r="D23" s="16">
         <v>27</v>
       </c>
-      <c r="E23" s="16">
+      <c r="E23" s="22">
         <v>337.29</v>
       </c>
-      <c r="F23" s="16">
+      <c r="F23" s="22">
         <v>468.13</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G23" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>64759.680000000008</v>
+      </c>
+      <c r="H23" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>130.83999999999997</v>
+      </c>
+      <c r="I23" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.38791544368347702</v>
+      </c>
+      <c r="J23" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" s="16" t="s">
         <v>311</v>
       </c>
@@ -8000,14 +8553,30 @@
       <c r="D24" s="16">
         <v>35</v>
       </c>
-      <c r="E24" s="16">
+      <c r="E24" s="22">
         <v>460.21</v>
       </c>
-      <c r="F24" s="16">
+      <c r="F24" s="22">
         <v>539.22</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G24" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>18868.61</v>
+      </c>
+      <c r="H24" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>79.010000000000048</v>
+      </c>
+      <c r="I24" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.17168249277503758</v>
+      </c>
+      <c r="J24" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" s="16" t="s">
         <v>312</v>
       </c>
@@ -8020,14 +8589,30 @@
       <c r="D25" s="16">
         <v>39</v>
       </c>
-      <c r="E25" s="16">
+      <c r="E25" s="22">
         <v>1322.63</v>
       </c>
-      <c r="F25" s="16">
+      <c r="F25" s="22">
         <v>1888.7</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G25" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>46292.05</v>
+      </c>
+      <c r="H25" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>566.06999999999994</v>
+      </c>
+      <c r="I25" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.42798817507541781</v>
+      </c>
+      <c r="J25" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>REORDER REQUIRED</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="16" t="s">
         <v>313</v>
       </c>
@@ -8040,14 +8625,30 @@
       <c r="D26" s="16">
         <v>41</v>
       </c>
-      <c r="E26" s="16">
+      <c r="E26" s="22">
         <v>512.17999999999995</v>
       </c>
-      <c r="F26" s="16">
+      <c r="F26" s="22">
         <v>754.23</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G26" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>52242.359999999993</v>
+      </c>
+      <c r="H26" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>242.05000000000007</v>
+      </c>
+      <c r="I26" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.47258776211488168</v>
+      </c>
+      <c r="J26" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="16" t="s">
         <v>314</v>
       </c>
@@ -8060,14 +8661,30 @@
       <c r="D27" s="16">
         <v>41</v>
       </c>
-      <c r="E27" s="16">
+      <c r="E27" s="22">
         <v>776.05</v>
       </c>
-      <c r="F27" s="16">
+      <c r="F27" s="22">
         <v>893.22</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G27" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>81485.25</v>
+      </c>
+      <c r="H27" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>117.17000000000007</v>
+      </c>
+      <c r="I27" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.15098253978480777</v>
+      </c>
+      <c r="J27" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="16" t="s">
         <v>316</v>
       </c>
@@ -8080,14 +8697,30 @@
       <c r="D28" s="16">
         <v>26</v>
       </c>
-      <c r="E28" s="16">
+      <c r="E28" s="22">
         <v>104.29</v>
       </c>
-      <c r="F28" s="16">
+      <c r="F28" s="22">
         <v>128.44999999999999</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G28" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>19293.650000000001</v>
+      </c>
+      <c r="H28" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>24.159999999999982</v>
+      </c>
+      <c r="I28" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.23166171253236151</v>
+      </c>
+      <c r="J28" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" s="16" t="s">
         <v>317</v>
       </c>
@@ -8100,14 +8733,30 @@
       <c r="D29" s="16">
         <v>27</v>
       </c>
-      <c r="E29" s="16">
+      <c r="E29" s="22">
         <v>674.22</v>
       </c>
-      <c r="F29" s="16">
+      <c r="F29" s="22">
         <v>995.35</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G29" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>113268.96</v>
+      </c>
+      <c r="H29" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>321.13</v>
+      </c>
+      <c r="I29" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.47629853756933938</v>
+      </c>
+      <c r="J29" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="16" t="s">
         <v>318</v>
       </c>
@@ -8120,14 +8769,30 @@
       <c r="D30" s="16">
         <v>50</v>
       </c>
-      <c r="E30" s="16">
+      <c r="E30" s="22">
         <v>1888.48</v>
       </c>
-      <c r="F30" s="16">
+      <c r="F30" s="22">
         <v>2373.98</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G30" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>73650.720000000001</v>
+      </c>
+      <c r="H30" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>485.5</v>
+      </c>
+      <c r="I30" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.25708506311954588</v>
+      </c>
+      <c r="J30" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>REORDER REQUIRED</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" s="16" t="s">
         <v>319</v>
       </c>
@@ -8140,14 +8805,30 @@
       <c r="D31" s="16">
         <v>39</v>
       </c>
-      <c r="E31" s="16">
+      <c r="E31" s="22">
         <v>263.41000000000003</v>
       </c>
-      <c r="F31" s="16">
+      <c r="F31" s="22">
         <v>308.41000000000003</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G31" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>23970.31</v>
+      </c>
+      <c r="H31" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>45</v>
+      </c>
+      <c r="I31" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.17083633878744162</v>
+      </c>
+      <c r="J31" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" s="16" t="s">
         <v>320</v>
       </c>
@@ -8160,14 +8841,30 @@
       <c r="D32" s="16">
         <v>43</v>
       </c>
-      <c r="E32" s="16">
+      <c r="E32" s="22">
         <v>1759.07</v>
       </c>
-      <c r="F32" s="16">
+      <c r="F32" s="22">
         <v>2276.62</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G32" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>263860.5</v>
+      </c>
+      <c r="H32" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>517.54999999999995</v>
+      </c>
+      <c r="I32" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.29421796744870865</v>
+      </c>
+      <c r="J32" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" s="16" t="s">
         <v>321</v>
       </c>
@@ -8180,14 +8877,30 @@
       <c r="D33" s="16">
         <v>24</v>
       </c>
-      <c r="E33" s="16">
+      <c r="E33" s="22">
         <v>1187.56</v>
       </c>
-      <c r="F33" s="16">
+      <c r="F33" s="22">
         <v>1361.95</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G33" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>66503.360000000001</v>
+      </c>
+      <c r="H33" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>174.3900000000001</v>
+      </c>
+      <c r="I33" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.14684731718818428</v>
+      </c>
+      <c r="J33" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" s="16" t="s">
         <v>322</v>
       </c>
@@ -8200,14 +8913,30 @@
       <c r="D34" s="16">
         <v>40</v>
       </c>
-      <c r="E34" s="16">
+      <c r="E34" s="22">
         <v>1026.1199999999999</v>
       </c>
-      <c r="F34" s="16">
+      <c r="F34" s="22">
         <v>1536.42</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G34" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>64645.55999999999</v>
+      </c>
+      <c r="H34" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>510.30000000000018</v>
+      </c>
+      <c r="I34" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.4973102561103967</v>
+      </c>
+      <c r="J34" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" s="16" t="s">
         <v>324</v>
       </c>
@@ -8220,14 +8949,30 @@
       <c r="D35" s="16">
         <v>45</v>
       </c>
-      <c r="E35" s="16">
+      <c r="E35" s="22">
         <v>1774.37</v>
       </c>
-      <c r="F35" s="16">
+      <c r="F35" s="22">
         <v>2343.67</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G35" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>46133.619999999995</v>
+      </c>
+      <c r="H35" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>569.30000000000018</v>
+      </c>
+      <c r="I35" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.3208462721980197</v>
+      </c>
+      <c r="J35" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>REORDER REQUIRED</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" s="16" t="s">
         <v>325</v>
       </c>
@@ -8240,14 +8985,30 @@
       <c r="D36" s="16">
         <v>34</v>
       </c>
-      <c r="E36" s="16">
+      <c r="E36" s="22">
         <v>2433.2199999999998</v>
       </c>
-      <c r="F36" s="16">
+      <c r="F36" s="22">
         <v>3067.33</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G36" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>92462.359999999986</v>
+      </c>
+      <c r="H36" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>634.11000000000013</v>
+      </c>
+      <c r="I36" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.26060528846549025</v>
+      </c>
+      <c r="J36" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" s="16" t="s">
         <v>326</v>
       </c>
@@ -8260,14 +9021,30 @@
       <c r="D37" s="16">
         <v>22</v>
       </c>
-      <c r="E37" s="16">
+      <c r="E37" s="22">
         <v>612.16</v>
       </c>
-      <c r="F37" s="16">
+      <c r="F37" s="22">
         <v>789.72</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G37" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>107128</v>
+      </c>
+      <c r="H37" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>177.56000000000006</v>
+      </c>
+      <c r="I37" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.29005488761108217</v>
+      </c>
+      <c r="J37" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" s="16" t="s">
         <v>327</v>
       </c>
@@ -8280,14 +9057,30 @@
       <c r="D38" s="16">
         <v>32</v>
       </c>
-      <c r="E38" s="16">
+      <c r="E38" s="22">
         <v>2099.98</v>
       </c>
-      <c r="F38" s="16">
+      <c r="F38" s="22">
         <v>2450.92</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G38" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>270897.42</v>
+      </c>
+      <c r="H38" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>350.94000000000005</v>
+      </c>
+      <c r="I38" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.16711587729406949</v>
+      </c>
+      <c r="J38" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" s="16" t="s">
         <v>328</v>
       </c>
@@ -8300,14 +9093,30 @@
       <c r="D39" s="16">
         <v>37</v>
       </c>
-      <c r="E39" s="16">
+      <c r="E39" s="22">
         <v>1496.14</v>
       </c>
-      <c r="F39" s="16">
+      <c r="F39" s="22">
         <v>1707.09</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G39" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>83783.840000000011</v>
+      </c>
+      <c r="H39" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>210.94999999999982</v>
+      </c>
+      <c r="I39" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.14099616346063859</v>
+      </c>
+      <c r="J39" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" s="16" t="s">
         <v>329</v>
       </c>
@@ -8320,14 +9129,30 @@
       <c r="D40" s="16">
         <v>32</v>
       </c>
-      <c r="E40" s="16">
+      <c r="E40" s="22">
         <v>517.16999999999996</v>
       </c>
-      <c r="F40" s="16">
+      <c r="F40" s="22">
         <v>593.35</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G40" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>10860.57</v>
+      </c>
+      <c r="H40" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>76.180000000000064</v>
+      </c>
+      <c r="I40" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.14730166096254629</v>
+      </c>
+      <c r="J40" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>REORDER REQUIRED</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" s="16" t="s">
         <v>330</v>
       </c>
@@ -8340,14 +9165,30 @@
       <c r="D41" s="16">
         <v>23</v>
       </c>
-      <c r="E41" s="16">
+      <c r="E41" s="22">
         <v>1419.91</v>
       </c>
-      <c r="F41" s="16">
+      <c r="F41" s="22">
         <v>1644.02</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G41" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>180328.57</v>
+      </c>
+      <c r="H41" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>224.1099999999999</v>
+      </c>
+      <c r="I41" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.15783394722200694</v>
+      </c>
+      <c r="J41" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" s="16" t="s">
         <v>331</v>
       </c>
@@ -8360,14 +9201,30 @@
       <c r="D42" s="16">
         <v>49</v>
       </c>
-      <c r="E42" s="16">
+      <c r="E42" s="22">
         <v>1790.94</v>
       </c>
-      <c r="F42" s="16">
+      <c r="F42" s="22">
         <v>2323.16</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G42" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>125365.8</v>
+      </c>
+      <c r="H42" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>532.2199999999998</v>
+      </c>
+      <c r="I42" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.29717355131941875</v>
+      </c>
+      <c r="J42" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" s="16" t="s">
         <v>332</v>
       </c>
@@ -8380,14 +9237,30 @@
       <c r="D43" s="16">
         <v>44</v>
       </c>
-      <c r="E43" s="16">
+      <c r="E43" s="22">
         <v>399.67</v>
       </c>
-      <c r="F43" s="16">
+      <c r="F43" s="22">
         <v>493.8</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G43" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>37968.65</v>
+      </c>
+      <c r="H43" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>94.13</v>
+      </c>
+      <c r="I43" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.23551930342532587</v>
+      </c>
+      <c r="J43" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" s="16" t="s">
         <v>333</v>
       </c>
@@ -8400,14 +9273,30 @@
       <c r="D44" s="16">
         <v>15</v>
       </c>
-      <c r="E44" s="16">
+      <c r="E44" s="22">
         <v>2270.09</v>
       </c>
-      <c r="F44" s="16">
+      <c r="F44" s="22">
         <v>3125.82</v>
       </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G44" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>195227.74000000002</v>
+      </c>
+      <c r="H44" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>855.73</v>
+      </c>
+      <c r="I44" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.37695862278588071</v>
+      </c>
+      <c r="J44" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45" s="16" t="s">
         <v>335</v>
       </c>
@@ -8420,14 +9309,30 @@
       <c r="D45" s="16">
         <v>30</v>
       </c>
-      <c r="E45" s="16">
+      <c r="E45" s="22">
         <v>2280.98</v>
       </c>
-      <c r="F45" s="16">
+      <c r="F45" s="22">
         <v>3040.92</v>
       </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G45" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>161949.57999999999</v>
+      </c>
+      <c r="H45" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>759.94</v>
+      </c>
+      <c r="I45" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.33316381555296409</v>
+      </c>
+      <c r="J45" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" s="16" t="s">
         <v>336</v>
       </c>
@@ -8440,14 +9345,30 @@
       <c r="D46" s="16">
         <v>25</v>
       </c>
-      <c r="E46" s="16">
+      <c r="E46" s="22">
         <v>1731.67</v>
       </c>
-      <c r="F46" s="16">
+      <c r="F46" s="22">
         <v>2345.9499999999998</v>
       </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G46" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>57145.11</v>
+      </c>
+      <c r="H46" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>614.27999999999975</v>
+      </c>
+      <c r="I46" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.35473271466272427</v>
+      </c>
+      <c r="J46" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" s="16" t="s">
         <v>337</v>
       </c>
@@ -8460,14 +9381,30 @@
       <c r="D47" s="16">
         <v>39</v>
       </c>
-      <c r="E47" s="16">
+      <c r="E47" s="22">
         <v>615.1</v>
       </c>
-      <c r="F47" s="16">
+      <c r="F47" s="22">
         <v>872.64</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G47" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>74427.100000000006</v>
+      </c>
+      <c r="H47" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>257.53999999999996</v>
+      </c>
+      <c r="I47" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.41869614696797264</v>
+      </c>
+      <c r="J47" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48" s="16" t="s">
         <v>339</v>
       </c>
@@ -8480,14 +9417,30 @@
       <c r="D48" s="16">
         <v>12</v>
       </c>
-      <c r="E48" s="16">
+      <c r="E48" s="22">
         <v>1606.36</v>
       </c>
-      <c r="F48" s="16">
+      <c r="F48" s="22">
         <v>1986.83</v>
       </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G48" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>287538.44</v>
+      </c>
+      <c r="H48" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>380.47</v>
+      </c>
+      <c r="I48" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.23685226225752637</v>
+      </c>
+      <c r="J48" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A49" s="16" t="s">
         <v>340</v>
       </c>
@@ -8500,14 +9453,30 @@
       <c r="D49" s="16">
         <v>44</v>
       </c>
-      <c r="E49" s="16">
+      <c r="E49" s="22">
         <v>1425.04</v>
       </c>
-      <c r="F49" s="16">
+      <c r="F49" s="22">
         <v>1716.14</v>
       </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G49" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>106878</v>
+      </c>
+      <c r="H49" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>291.10000000000014</v>
+      </c>
+      <c r="I49" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.20427496772020445</v>
+      </c>
+      <c r="J49" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50" s="16" t="s">
         <v>341</v>
       </c>
@@ -8520,14 +9489,30 @@
       <c r="D50" s="16">
         <v>19</v>
       </c>
-      <c r="E50" s="16">
+      <c r="E50" s="22">
         <v>1481.18</v>
       </c>
-      <c r="F50" s="16">
+      <c r="F50" s="22">
         <v>1660.13</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G50" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>223658.18000000002</v>
+      </c>
+      <c r="H50" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>178.95000000000005</v>
+      </c>
+      <c r="I50" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.12081583602263063</v>
+      </c>
+      <c r="J50" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A51" s="16" t="s">
         <v>343</v>
       </c>
@@ -8540,14 +9525,30 @@
       <c r="D51" s="16">
         <v>50</v>
       </c>
-      <c r="E51" s="16">
+      <c r="E51" s="22">
         <v>2480.2600000000002</v>
       </c>
-      <c r="F51" s="16">
+      <c r="F51" s="22">
         <v>2854.49</v>
       </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G51" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>456367.84</v>
+      </c>
+      <c r="H51" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>374.22999999999956</v>
+      </c>
+      <c r="I51" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.1508833751300265</v>
+      </c>
+      <c r="J51" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A52" s="16" t="s">
         <v>309</v>
       </c>
@@ -8560,11 +9561,27 @@
       <c r="D52" s="16">
         <v>27</v>
       </c>
-      <c r="E52" s="16">
+      <c r="E52" s="22">
         <v>337.29</v>
       </c>
-      <c r="F52" s="16">
+      <c r="F52" s="22">
         <v>468.13</v>
+      </c>
+      <c r="G52" s="22">
+        <f>InventoryTable[[#This Row],[CurrentStock]] * InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>64759.680000000008</v>
+      </c>
+      <c r="H52" s="22">
+        <f>InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>130.83999999999997</v>
+      </c>
+      <c r="I52" s="24">
+        <f>(InventoryTable[[#This Row],[SellingPrice]] - InventoryTable[[#This Row],[CostPerUnit]]) / InventoryTable[[#This Row],[CostPerUnit]]</f>
+        <v>0.38791544368347702</v>
+      </c>
+      <c r="J52" s="22" t="str">
+        <f>IF(InventoryTable[[#This Row],[CurrentStock]] &lt;= InventoryTable[[#This Row],[ReorderLevel]], "REORDER REQUIRED", "IN STOCK")</f>
+        <v>IN STOCK</v>
       </c>
     </row>
   </sheetData>

</xml_diff>